<commit_message>
Creación de módulo de lectura de correos de Gmail y modificación del fichero de configuración (Config.xlsx)
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alicia LV\Downloads\REF_plantilla\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frand\Documents\UiPath\REF_RPAw\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30566933-CC83-4638-BFB7-35C9390415D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0218EC-CF76-4F0A-9557-9D0CEBA21BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -152,12 +152,6 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>Trabajadores</t>
-  </si>
-  <si>
-    <t>aliciafilosofiamn@gmail.com's workspace</t>
-  </si>
-  <si>
     <t>OrchestratorQueueName</t>
   </si>
   <si>
@@ -170,10 +164,16 @@
     <t>ListKill</t>
   </si>
   <si>
-    <t>MiProceso</t>
-  </si>
-  <si>
     <t>EXCEL</t>
+  </si>
+  <si>
+    <t>CorreosGmail</t>
+  </si>
+  <si>
+    <t>grupodeadpoolgeneration@gmail.com's workspace</t>
+  </si>
+  <si>
+    <t>RPAw</t>
   </si>
 </sst>
 </file>
@@ -253,7 +253,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -550,12 +550,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.54296875" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.453125" customWidth="1"/>
-    <col min="4" max="26" width="8.6328125" customWidth="1"/>
+    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -594,33 +594,33 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.5">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="29">
+    <row r="5" spans="1:26" ht="30">
       <c r="A5" t="s">
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -631,18 +631,18 @@
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1643,12 +1643,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.453125" customWidth="1"/>
-    <col min="4" max="26" width="8.6328125" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1685,7 +1685,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="29">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.5">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -1810,7 +1810,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="29">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -2801,12 +2801,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.90625" customWidth="1"/>
-    <col min="2" max="2" width="30.08984375" customWidth="1"/>
-    <col min="3" max="3" width="60.36328125" customWidth="1"/>
-    <col min="4" max="26" width="65.453125" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.42578125" customWidth="1"/>
+    <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Actualizado módulo 'LoginChatGPT' y empezado a trabajar con los filtros de Arcanoe
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Documents\Documentos\UiPath\RPAw\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Documents\Documentos\UiPath\RPAw_geles_v2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2382FF-CE96-4FBF-8432-BE7F9B0E954F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C894E992-BDDE-4F66-B2D1-0265C4053292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20610" yWindow="1980" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -179,13 +179,13 @@
     <t>URLChatGPT</t>
   </si>
   <si>
-    <t>https://chatgpt.com/es</t>
-  </si>
-  <si>
-    <t>El usuario proporcionado no es válido o no existe</t>
-  </si>
-  <si>
     <t>SL-01</t>
+  </si>
+  <si>
+    <t>El usuario o contraseña proporcionado no es válido o no existe</t>
+  </si>
+  <si>
+    <t>https://chatgpt.com/auth/login</t>
   </si>
 </sst>
 </file>
@@ -237,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -247,6 +247,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,7 +566,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.54296875" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
+    <col min="2" max="2" width="54.36328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="81.453125" customWidth="1"/>
     <col min="4" max="26" width="8.54296875" customWidth="1"/>
   </cols>
@@ -662,14 +663,14 @@
       <c r="A12" t="s">
         <v>50</v>
       </c>
-      <c r="B12" t="s">
-        <v>51</v>
+      <c r="B12" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Integración de módulo de extracción de datos de mascotas.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frand\Documents\UiPath\RPAw\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A65C784-35F8-43D6-85F1-308CBEFA5D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD01C4A6-C7A3-4D6E-9D4B-12F39F141D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -191,13 +191,13 @@
     <t>SL-01: Error de login Chat GPT</t>
   </si>
   <si>
-    <t xml:space="preserve">Te voy a pasar un texto. Necesito que compruebes si hace referencia a algún animal y, en caso afirmativo, extraigas los siguientes criterios de búsqueda. Si el texto menciona un animal pero no contiene información clara sobre algún criterio, asigna los valores correspondientes a los campos faltantes como "". Si el texto no hace referencia a ningún animal o no está relacionado con la adopción, acogida o apadrinamiento de un animal, responde exclusivamente con "No es válido". Los criterios de búsqueda son: Tipo de mascota: Perro, Gato o Animal exótico. Sexo: Macho o Hembra. Edad: Cachorro, Cachorrito, Joven, Adulto, Veterano, Abuelo. Tamaño: Mini, Pequeño, Mediano, Grande, Gigante. Entrega la información en formato diccionario clave-valor. Formato de respuesta: { 'Tipo_mascota': valor, 'Sexo': valor, 'Edad': valor, 'Tamaño': valor } Si no hay referencias claras a los animales ni a la adopción o apadrinamiento, devuelve: "No es válido". El texto es: </t>
-  </si>
-  <si>
     <t>URLArcadeNoe</t>
   </si>
   <si>
     <t>https://arcadenoe.org/</t>
+  </si>
+  <si>
+    <t>Te voy a pasar un texto. Necesito que compruebes si hace referencia a algún animal y, en caso afirmativo, extraigas los siguientes criterios de búsqueda. Si el texto menciona un animal pero no contiene información clara sobre algún criterio, asigna los valores correspondientes a los campos faltantes como "". Si el texto no hace referencia a ningún animal o no está relacionado con la adopción, acogida o apadrinamiento de un animal, responde exclusivamente con "No es válido". Los criterios de búsqueda son: Tipo de mascota: Perro, Gato o Animal exótico. Sexo: Macho o Hembra. Edad: Cachorro, Cachorrito, Joven, Adulto, Veterano, Abuelo. Tamaño: Mini, Pequeño, Mediano, Grande, Gigante. Entrega la información en formato diccionario clave-valor en texto plano. Formato de respuesta: { 'Tipo_mascota': valor, 'Sexo': valor, 'Edad': valor, 'Tamaño': valor } Si no hay referencias claras a los animales ni a la adopción o apadrinamiento, devuelve: "No es válido". El texto es:</t>
   </si>
 </sst>
 </file>
@@ -680,10 +680,10 @@
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
         <v>56</v>
-      </c>
-      <c r="B13" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
@@ -691,7 +691,7 @@
         <v>53</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Corrección error popup e implementación cierre de aplicaciones.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frand\Documents\UiPath\RPAw\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD01C4A6-C7A3-4D6E-9D4B-12F39F141D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D5CA92-5A37-4456-85E3-7AA2095881E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>Name</t>
   </si>
@@ -164,9 +164,6 @@
     <t>ListKill</t>
   </si>
   <si>
-    <t>EXCEL</t>
-  </si>
-  <si>
     <t>CorreosGmail</t>
   </si>
   <si>
@@ -198,6 +195,15 @@
   </si>
   <si>
     <t>Te voy a pasar un texto. Necesito que compruebes si hace referencia a algún animal y, en caso afirmativo, extraigas los siguientes criterios de búsqueda. Si el texto menciona un animal pero no contiene información clara sobre algún criterio, asigna los valores correspondientes a los campos faltantes como "". Si el texto no hace referencia a ningún animal o no está relacionado con la adopción, acogida o apadrinamiento de un animal, responde exclusivamente con "No es válido". Los criterios de búsqueda son: Tipo de mascota: Perro, Gato o Animal exótico. Sexo: Macho o Hembra. Edad: Cachorro, Cachorrito, Joven, Adulto, Veterano, Abuelo. Tamaño: Mini, Pequeño, Mediano, Grande, Gigante. Entrega la información en formato diccionario clave-valor en texto plano. Formato de respuesta: { 'Tipo_mascota': valor, 'Sexo': valor, 'Edad': valor, 'Tamaño': valor } Si no hay referencias claras a los animales ni a la adopción o apadrinamiento, devuelve: "No es válido". El texto es:</t>
+  </si>
+  <si>
+    <t>ErrorSesionGoogle</t>
+  </si>
+  <si>
+    <t>Error en el inicio de sesión con Google</t>
+  </si>
+  <si>
+    <t>EXCEL;CHROME</t>
   </si>
 </sst>
 </file>
@@ -573,7 +579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -621,7 +627,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -632,7 +638,7 @@
         <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>30</v>
@@ -644,7 +650,7 @@
         <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -665,60 +671,67 @@
       <c r="A10" t="s">
         <v>45</v>
       </c>
-      <c r="B10" t="s">
-        <v>46</v>
+      <c r="B10" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" t="s">
         <v>50</v>
-      </c>
-      <c r="B12" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
         <v>55</v>
-      </c>
-      <c r="B13" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="17" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1686,6 +1699,7 @@
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
+    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cambios parámetros Process e implementación de BusinessException.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frand\Documents\UiPath\RPAw\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D5CA92-5A37-4456-85E3-7AA2095881E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97074A7-E65B-47AA-BD0C-28A82BCCF14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
   <si>
     <t>Name</t>
   </si>
@@ -195,12 +195,6 @@
   </si>
   <si>
     <t>Te voy a pasar un texto. Necesito que compruebes si hace referencia a algún animal y, en caso afirmativo, extraigas los siguientes criterios de búsqueda. Si el texto menciona un animal pero no contiene información clara sobre algún criterio, asigna los valores correspondientes a los campos faltantes como "". Si el texto no hace referencia a ningún animal o no está relacionado con la adopción, acogida o apadrinamiento de un animal, responde exclusivamente con "No es válido". Los criterios de búsqueda son: Tipo de mascota: Perro, Gato o Animal exótico. Sexo: Macho o Hembra. Edad: Cachorro, Cachorrito, Joven, Adulto, Veterano, Abuelo. Tamaño: Mini, Pequeño, Mediano, Grande, Gigante. Entrega la información en formato diccionario clave-valor en texto plano. Formato de respuesta: { 'Tipo_mascota': valor, 'Sexo': valor, 'Edad': valor, 'Tamaño': valor } Si no hay referencias claras a los animales ni a la adopción o apadrinamiento, devuelve: "No es válido". El texto es:</t>
-  </si>
-  <si>
-    <t>ErrorSesionGoogle</t>
-  </si>
-  <si>
-    <t>Error en el inicio de sesión con Google</t>
   </si>
   <si>
     <t>EXCEL;CHROME</t>
@@ -579,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -672,7 +666,7 @@
         <v>45</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -703,35 +697,28 @@
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="17" ht="14.25" customHeight="1"/>
+    <row r="18" ht="14.25" customHeight="1"/>
+    <row r="19" ht="14.25" customHeight="1"/>
+    <row r="20" ht="14.25" customHeight="1"/>
+    <row r="21" ht="14.25" customHeight="1"/>
+    <row r="22" ht="14.25" customHeight="1"/>
+    <row r="23" ht="14.25" customHeight="1"/>
+    <row r="24" ht="14.25" customHeight="1"/>
+    <row r="25" ht="14.25" customHeight="1"/>
+    <row r="26" ht="14.25" customHeight="1"/>
+    <row r="27" ht="14.25" customHeight="1"/>
+    <row r="28" ht="14.25" customHeight="1"/>
+    <row r="29" ht="14.25" customHeight="1"/>
+    <row r="30" ht="14.25" customHeight="1"/>
+    <row r="31" ht="14.25" customHeight="1"/>
+    <row r="32" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1699,7 +1686,6 @@
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Integración de envío de correos, mejoras y corrección de errores.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frand\Documents\UiPath\RPAw\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97074A7-E65B-47AA-BD0C-28A82BCCF14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B71B8F3-3EB0-42DE-AD01-837F2E9F27BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="78">
   <si>
     <t>Name</t>
   </si>
@@ -179,9 +179,6 @@
     <t>https://chatgpt.com/auth/login</t>
   </si>
   <si>
-    <t>SL01</t>
-  </si>
-  <si>
     <t>PromptChatGPT</t>
   </si>
   <si>
@@ -198,13 +195,103 @@
   </si>
   <si>
     <t>EXCEL;CHROME</t>
+  </si>
+  <si>
+    <t>SL-02</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">SL-02: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>No existen mascotas</t>
+    </r>
+  </si>
+  <si>
+    <t>SL01AsuntoCorreo</t>
+  </si>
+  <si>
+    <t>SL02AsuntoCorreo</t>
+  </si>
+  <si>
+    <t>SL01CuerpoCorreo</t>
+  </si>
+  <si>
+    <t>SL02CuerpoCorreo</t>
+  </si>
+  <si>
+    <t>Hola, 
+RPAw ha detectado el siguiente error:
+SL-01: No se pudo iniciar sesión en Chat GPT.</t>
+  </si>
+  <si>
+    <t>SL-01</t>
+  </si>
+  <si>
+    <t>CorreoInterno</t>
+  </si>
+  <si>
+    <t>grupodeadpoolgeneration@gmail.com</t>
+  </si>
+  <si>
+    <t>Arca de Noé responde a su consulta</t>
+  </si>
+  <si>
+    <t>RPAw ALERTA - SL-01: Login no válido</t>
+  </si>
+  <si>
+    <t>RutaFicherosSalida</t>
+  </si>
+  <si>
+    <t>Output\Ficheros</t>
+  </si>
+  <si>
+    <t>Listado de mascotas coincidentes</t>
+  </si>
+  <si>
+    <t>Hola,
+En primer lugar, te agradecemos que te hayas puesto en contacto con Arca de Noé. 
+Lamentablemente, tras valorar tu solicitud no disponemos en este momento de mascotas que cumplan con los criterios que nos has solicitado. 
+No obstante, disponemos de muchas otras que están deseando ser acogidas. 
+Te animamos a que visites nuestra web y les des una oportunidad. ¡Ellas te necesitan!
+Si lo prefieres puedes volver a respondernos a este email o contactar con nosotros en el teléfono abajo indicado.
+¡¡Gracias y un abrazo!!
+Arca de Noé
+Tlf: 659 30 56 89</t>
+  </si>
+  <si>
+    <t>AsuntoCorreoResultados</t>
+  </si>
+  <si>
+    <t>CuerpoCorreoResultados</t>
+  </si>
+  <si>
+    <t>RutaPlantillas</t>
+  </si>
+  <si>
+    <t>Hola,
+Queremos agradecerte que te hayas puesto en contacto con Arca de Noé. 
+A continuación adjuntamos un fichero excel con un listado de candidatos coincidentes y fichas detalladas de cada uno de ellos.
+¡¡¡Esperamos tener pronto noticias tuyas!!!
+Un saludo.
+Arca de Noé
+Tlf: 659 30 56 89</t>
+  </si>
+  <si>
+    <t>Data\Input</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -223,6 +310,13 @@
       <charset val="128"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -249,7 +343,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -259,6 +353,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z1002"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -666,7 +761,7 @@
         <v>45</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -680,45 +775,120 @@
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
         <v>54</v>
-      </c>
-      <c r="B13" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>56</v>
-      </c>
     </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" t="s">
-        <v>53</v>
-      </c>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="5"/>
     </row>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="5"/>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" s="5"/>
+    </row>
+    <row r="30" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B30" s="5"/>
+    </row>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1686,6 +1856,9 @@
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
+    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="1001" ht="14.25" customHeight="1"/>
+    <row r="1002" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Revisión y documentación del código.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\frand\Documents\UiPath\RPAw\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B71B8F3-3EB0-42DE-AD01-837F2E9F27BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B50A6BA-4B78-4A40-B7FF-3C1129CA7E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="79">
   <si>
     <t>Name</t>
   </si>
@@ -285,6 +285,9 @@
   </si>
   <si>
     <t>Data\Input</t>
+  </si>
+  <si>
+    <t>Proceso que se finalizarán. Van separados por ;</t>
   </si>
 </sst>
 </file>
@@ -762,6 +765,9 @@
       </c>
       <c r="B10" s="2" t="s">
         <v>56</v>
+      </c>
+      <c r="C10" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>